<commit_message>
Added Panel of ref-sites in ordinated env-spaces.
</commit_message>
<xml_diff>
--- a/results/02_taxa_assemblage/MRT_Method/cluster_classifier/tables/mrt_cp_table.xlsx
+++ b/results/02_taxa_assemblage/MRT_Method/cluster_classifier/tables/mrt_cp_table.xlsx
@@ -446,22 +446,22 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>xerror</t>
+          <t>CV error</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>xstd</t>
+          <t>CV std</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>xcv_lo</t>
+          <t>CV lo</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>xcv_hi</t>
+          <t>CV hi</t>
         </is>
       </c>
     </row>

</xml_diff>